<commit_message>
Prueba 2 (word con keys)
</commit_message>
<xml_diff>
--- a/Transfer_Answers/Inputs/Forms_Data.xlsx
+++ b/Transfer_Answers/Inputs/Forms_Data.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29917"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{487C11D7-6183-4410-8B82-33684D30D86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BBA3BF0-8595-42AD-ABA9-08DD52CBBC70}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{487C11D7-6183-4410-8B82-33684D30D86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B22F34AF-75E5-4F8F-9596-D624E1ACC622}"/>
   <bookViews>
     <workbookView xWindow="3240" yWindow="2076" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="44">
   <si>
     <t xml:space="preserve">profesor_guia </t>
   </si>
@@ -136,13 +136,43 @@
   </si>
   <si>
     <t>p13_no</t>
+  </si>
+  <si>
+    <t>nombre</t>
+  </si>
+  <si>
+    <t>rut</t>
+  </si>
+  <si>
+    <t>solicito</t>
+  </si>
+  <si>
+    <t>oing</t>
+  </si>
+  <si>
+    <t>26/204</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>ing</t>
+  </si>
+  <si>
+    <t>benja</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mmm"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -275,23 +305,74 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="40">
+  <dxfs count="43">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -750,7 +831,7 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="21" formatCode="dd/mmm"/>
+      <numFmt numFmtId="164" formatCode="dd/mmm"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -890,25 +971,6 @@
           <color indexed="64"/>
         </top>
       </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -916,6 +978,25 @@
           <color indexed="64"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -965,49 +1046,48 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{49004379-8959-4804-8411-638F21A2B811}" name="Tabla2" displayName="Tabla2" ref="A1:AI2" insertRow="1" totalsRowShown="0" headerRowDxfId="39" dataDxfId="37" headerRowBorderDxfId="38" tableBorderDxfId="36" totalsRowBorderDxfId="35">
-  <autoFilter ref="A1:AI2" xr:uid="{49004379-8959-4804-8411-638F21A2B811}"/>
-  <tableColumns count="35">
-    <tableColumn id="1" xr3:uid="{1BB3FF62-5FB4-4329-B41B-91C5CB718039}" name="profesor_guia " dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{7B9E9655-9D90-44EE-850C-202257B4F4F0}" name="titulo" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{D52AE646-FF35-45EC-8758-03C85DDB83AD}" name="modalidad" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{FFE233A2-8272-4BE6-923F-DE41EFF53853}" name="objetivo_general" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{37A58E33-97C0-4659-B2E9-932167611FF7}" name="objetivos_especificos" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{D2F46401-1025-4BC3-B06E-81AC6FA90F7C}" name="material_presupuesto" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{76DA7FF9-9CED-44C8-97B3-5BB7A3B32DB6}" name="requisitos_alumno" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{10BB6D6C-EB03-4BF1-9968-950E0BC62566}" name="fecha" dataDxfId="27"/>
-    <tableColumn id="9" xr3:uid="{598335C7-F48C-4354-8258-C674203051FD}" name="actividades_principales" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{045334EE-BC9F-427E-8A94-101D923CA495}" name="p1_si" dataDxfId="25"/>
-    <tableColumn id="11" xr3:uid="{51347BC5-59CC-4262-8BD0-990116224809}" name="p2_si" dataDxfId="24"/>
-    <tableColumn id="12" xr3:uid="{9C650AA7-729C-444D-8BB2-3868583362DB}" name="p3_si" dataDxfId="23"/>
-    <tableColumn id="13" xr3:uid="{C48B699B-44A2-432F-8CA0-8353B2EEFFF5}" name="p4_si" dataDxfId="22"/>
-    <tableColumn id="14" xr3:uid="{A8949987-D248-4F5A-928F-BFB01AA6D109}" name="p5_si" dataDxfId="21"/>
-    <tableColumn id="15" xr3:uid="{B087A3C0-321B-4A16-8FFA-C46A9FC1891B}" name="p6_si" dataDxfId="20"/>
-    <tableColumn id="16" xr3:uid="{E3B50787-59E8-42DB-A192-5DA51F2BE5C7}" name="p7_si" dataDxfId="19"/>
-    <tableColumn id="17" xr3:uid="{FD4835CA-FA39-460D-92F9-DE6BEDB86486}" name="p8_si" dataDxfId="18"/>
-    <tableColumn id="18" xr3:uid="{6FFD8438-3CB6-468B-AB46-01BD9AAC31E3}" name="p9_si" dataDxfId="17"/>
-    <tableColumn id="19" xr3:uid="{9575FF1B-E10F-4F4E-8D56-39AD053507AF}" name="p10_si" dataDxfId="16"/>
-    <tableColumn id="20" xr3:uid="{EBDAAB99-CAF2-4981-9AB2-AD84D0EC31BC}" name="p11_si" dataDxfId="15"/>
-    <tableColumn id="21" xr3:uid="{2B3439E6-35D8-4B80-8C3C-B3B02FDE4B18}" name="p12_si" dataDxfId="14"/>
-    <tableColumn id="22" xr3:uid="{9DBEACE7-6E7E-44F6-B916-BEC162450435}" name="p13_si" dataDxfId="13"/>
-    <tableColumn id="23" xr3:uid="{D81B8290-8921-4D69-9377-015676DBB2A3}" name="p1_no" dataDxfId="12"/>
-    <tableColumn id="24" xr3:uid="{885ECDD6-4FB9-4B60-816D-4734E9B83E91}" name="p2_no" dataDxfId="11"/>
-    <tableColumn id="25" xr3:uid="{4E29BBAC-4514-44AD-A96F-237D093E7EF9}" name="p3_no" dataDxfId="10"/>
-    <tableColumn id="26" xr3:uid="{E36BE3CA-E872-406B-BBDD-8F8EF27E7ECB}" name="p4_no" dataDxfId="9"/>
-    <tableColumn id="27" xr3:uid="{BEB8C10C-4139-46A0-97F9-EE4BFE76A8C4}" name="p5_no" dataDxfId="8"/>
-    <tableColumn id="28" xr3:uid="{7B6B2FBC-551C-447F-8B19-46955A728668}" name="p6_no" dataDxfId="7"/>
-    <tableColumn id="29" xr3:uid="{4D3D9DA6-284D-4774-AFD2-4CF3EF645A5C}" name="p7_no" dataDxfId="6"/>
-    <tableColumn id="30" xr3:uid="{7AFD40AA-0042-4154-A253-4DCC538704A9}" name="p8_no" dataDxfId="5"/>
-    <tableColumn id="31" xr3:uid="{E0C8EA75-1EC4-4E3C-9AAB-3AB47E6E0A2F}" name="p9_no" dataDxfId="4"/>
-    <tableColumn id="32" xr3:uid="{5C92C993-4B6F-4EF2-BD4F-67455BDA8A9B}" name="p10_no" dataDxfId="3"/>
-    <tableColumn id="33" xr3:uid="{F77ED6D2-9D4D-420B-91B0-BDB16DEED2F9}" name="p11_no" dataDxfId="2"/>
-    <tableColumn id="34" xr3:uid="{1BBAF427-78B8-45A7-8CFE-0E830B47FDF8}" name="p12_no" dataDxfId="1"/>
-    <tableColumn id="35" xr3:uid="{C16EA744-60FB-4022-981C-BECAC568CF4F}" name="p13_no" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{49004379-8959-4804-8411-638F21A2B811}" name="Tabla2" displayName="Tabla2" ref="A1:AL3" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41" headerRowBorderDxfId="39" tableBorderDxfId="40" totalsRowBorderDxfId="38">
+  <autoFilter ref="A1:AL3" xr:uid="{49004379-8959-4804-8411-638F21A2B811}"/>
+  <tableColumns count="38">
+    <tableColumn id="1" xr3:uid="{1BB3FF62-5FB4-4329-B41B-91C5CB718039}" name="profesor_guia " dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{7B9E9655-9D90-44EE-850C-202257B4F4F0}" name="titulo" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{D52AE646-FF35-45EC-8758-03C85DDB83AD}" name="modalidad" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{FFE233A2-8272-4BE6-923F-DE41EFF53853}" name="objetivo_general" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{37A58E33-97C0-4659-B2E9-932167611FF7}" name="objetivos_especificos" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{D2F46401-1025-4BC3-B06E-81AC6FA90F7C}" name="material_presupuesto" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{76DA7FF9-9CED-44C8-97B3-5BB7A3B32DB6}" name="requisitos_alumno" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{10BB6D6C-EB03-4BF1-9968-950E0BC62566}" name="fecha" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{598335C7-F48C-4354-8258-C674203051FD}" name="actividades_principales" dataDxfId="29"/>
+    <tableColumn id="10" xr3:uid="{045334EE-BC9F-427E-8A94-101D923CA495}" name="p1_si" dataDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{51347BC5-59CC-4262-8BD0-990116224809}" name="p2_si" dataDxfId="27"/>
+    <tableColumn id="12" xr3:uid="{9C650AA7-729C-444D-8BB2-3868583362DB}" name="p3_si" dataDxfId="26"/>
+    <tableColumn id="13" xr3:uid="{C48B699B-44A2-432F-8CA0-8353B2EEFFF5}" name="p4_si" dataDxfId="25"/>
+    <tableColumn id="14" xr3:uid="{A8949987-D248-4F5A-928F-BFB01AA6D109}" name="p5_si" dataDxfId="24"/>
+    <tableColumn id="15" xr3:uid="{B087A3C0-321B-4A16-8FFA-C46A9FC1891B}" name="p6_si" dataDxfId="23"/>
+    <tableColumn id="16" xr3:uid="{E3B50787-59E8-42DB-A192-5DA51F2BE5C7}" name="p7_si" dataDxfId="22"/>
+    <tableColumn id="17" xr3:uid="{FD4835CA-FA39-460D-92F9-DE6BEDB86486}" name="p8_si" dataDxfId="21"/>
+    <tableColumn id="18" xr3:uid="{6FFD8438-3CB6-468B-AB46-01BD9AAC31E3}" name="p9_si" dataDxfId="20"/>
+    <tableColumn id="19" xr3:uid="{9575FF1B-E10F-4F4E-8D56-39AD053507AF}" name="p10_si" dataDxfId="19"/>
+    <tableColumn id="20" xr3:uid="{EBDAAB99-CAF2-4981-9AB2-AD84D0EC31BC}" name="p11_si" dataDxfId="18"/>
+    <tableColumn id="21" xr3:uid="{2B3439E6-35D8-4B80-8C3C-B3B02FDE4B18}" name="p12_si" dataDxfId="17"/>
+    <tableColumn id="22" xr3:uid="{9DBEACE7-6E7E-44F6-B916-BEC162450435}" name="p13_si" dataDxfId="16"/>
+    <tableColumn id="23" xr3:uid="{D81B8290-8921-4D69-9377-015676DBB2A3}" name="p1_no" dataDxfId="15"/>
+    <tableColumn id="24" xr3:uid="{885ECDD6-4FB9-4B60-816D-4734E9B83E91}" name="p2_no" dataDxfId="14"/>
+    <tableColumn id="25" xr3:uid="{4E29BBAC-4514-44AD-A96F-237D093E7EF9}" name="p3_no" dataDxfId="13"/>
+    <tableColumn id="26" xr3:uid="{E36BE3CA-E872-406B-BBDD-8F8EF27E7ECB}" name="p4_no" dataDxfId="12"/>
+    <tableColumn id="27" xr3:uid="{BEB8C10C-4139-46A0-97F9-EE4BFE76A8C4}" name="p5_no" dataDxfId="11"/>
+    <tableColumn id="28" xr3:uid="{7B6B2FBC-551C-447F-8B19-46955A728668}" name="p6_no" dataDxfId="10"/>
+    <tableColumn id="29" xr3:uid="{4D3D9DA6-284D-4774-AFD2-4CF3EF645A5C}" name="p7_no" dataDxfId="9"/>
+    <tableColumn id="30" xr3:uid="{7AFD40AA-0042-4154-A253-4DCC538704A9}" name="p8_no" dataDxfId="8"/>
+    <tableColumn id="31" xr3:uid="{E0C8EA75-1EC4-4E3C-9AAB-3AB47E6E0A2F}" name="p9_no" dataDxfId="7"/>
+    <tableColumn id="32" xr3:uid="{5C92C993-4B6F-4EF2-BD4F-67455BDA8A9B}" name="p10_no" dataDxfId="6"/>
+    <tableColumn id="33" xr3:uid="{F77ED6D2-9D4D-420B-91B0-BDB16DEED2F9}" name="p11_no" dataDxfId="5"/>
+    <tableColumn id="34" xr3:uid="{1BBAF427-78B8-45A7-8CFE-0E830B47FDF8}" name="p12_no" dataDxfId="4"/>
+    <tableColumn id="35" xr3:uid="{C16EA744-60FB-4022-981C-BECAC568CF4F}" name="p13_no" dataDxfId="3"/>
+    <tableColumn id="36" xr3:uid="{997B0DC7-4EC6-43A0-B8F1-1EBDE4C902D5}" name="nombre" dataDxfId="2"/>
+    <tableColumn id="37" xr3:uid="{F334C1D3-22AD-4E2A-B58D-887C17BA1217}" name="rut" dataDxfId="1"/>
+    <tableColumn id="38" xr3:uid="{C2681029-970B-4E9B-8D16-E98AEBDD233C}" name="solicito" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1276,27 +1356,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AL8"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="21.5546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" style="1" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="19" customWidth="1"/>
-    <col min="8" max="8" width="21.33203125" customWidth="1"/>
-    <col min="9" max="9" width="23.109375" customWidth="1"/>
-    <col min="10" max="15" width="7.33203125" customWidth="1"/>
-    <col min="16" max="16" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="7.33203125" customWidth="1"/>
-    <col min="19" max="31" width="8.33203125" customWidth="1"/>
-    <col min="32" max="35" width="9.33203125" customWidth="1"/>
-    <col min="36" max="37" width="6.5546875" customWidth="1"/>
+    <col min="8" max="8" width="21.28515625" customWidth="1"/>
+    <col min="9" max="9" width="23.140625" customWidth="1"/>
+    <col min="10" max="15" width="7.28515625" customWidth="1"/>
+    <col min="16" max="16" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="7.28515625" customWidth="1"/>
+    <col min="19" max="31" width="8.28515625" customWidth="1"/>
+    <col min="32" max="35" width="9.28515625" customWidth="1"/>
+    <col min="36" max="37" width="6.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:38">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1402,72 +1482,263 @@
       <c r="AI1" s="4" t="s">
         <v>34</v>
       </c>
+      <c r="AJ1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="3" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
+    <row r="2" spans="1:38" ht="15">
+      <c r="A2" s="5">
+        <v>215125</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="6">
+        <v>42662</v>
+      </c>
+      <c r="D2" s="6">
+        <v>326236</v>
+      </c>
+      <c r="E2" s="6">
+        <v>6457347</v>
+      </c>
+      <c r="F2" s="6">
+        <v>613671</v>
+      </c>
+      <c r="G2" s="6">
+        <v>371613</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="6">
+        <v>427236</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
-      <c r="X2" s="6"/>
-      <c r="Y2" s="6"/>
-      <c r="Z2" s="6"/>
-      <c r="AA2" s="6"/>
+      <c r="P2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="S2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="W2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="X2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA2" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="AB2" s="6"/>
-      <c r="AC2" s="6"/>
-      <c r="AD2" s="6"/>
-      <c r="AE2" s="6"/>
-      <c r="AF2" s="6"/>
-      <c r="AG2" s="6"/>
-      <c r="AH2" s="6"/>
-      <c r="AI2" s="8"/>
+      <c r="AC2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AD2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="AF2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="AI2" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="AJ2" s="6"/>
+      <c r="AK2" s="6"/>
+      <c r="AL2" s="6"/>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A3"/>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
-      <c r="E3"/>
+    <row r="3" spans="1:38" ht="15">
+      <c r="A3" s="5">
+        <v>2412512</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="6">
+        <v>214214</v>
+      </c>
+      <c r="D3" s="6">
+        <v>521512</v>
+      </c>
+      <c r="E3" s="6">
+        <v>251521</v>
+      </c>
+      <c r="F3" s="6">
+        <v>31513</v>
+      </c>
+      <c r="G3" s="6">
+        <v>21521</v>
+      </c>
+      <c r="H3" s="7">
+        <v>1232124</v>
+      </c>
+      <c r="I3" s="6">
+        <v>215125</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="V3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="W3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="X3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="AD3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="AE3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AF3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AG3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AI3" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="AJ3" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AK3" s="6">
+        <v>12421</v>
+      </c>
+      <c r="AL3" s="6" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:38" ht="15">
       <c r="A4"/>
       <c r="B4"/>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:38" ht="15">
       <c r="A5"/>
       <c r="B5"/>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:38" ht="15">
       <c r="A6"/>
       <c r="B6"/>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
     </row>
+    <row r="7" spans="1:38" ht="15">
+      <c r="A7"/>
+      <c r="B7"/>
+      <c r="C7"/>
+      <c r="D7"/>
+      <c r="E7"/>
+    </row>
+    <row r="8" spans="1:38" ht="15"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>